<commit_message>
xue tiao follow player
</commit_message>
<xml_diff>
--- a/Assets/Configs/GameModifiers.xlsx
+++ b/Assets/Configs/GameModifiers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\minigame\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FEC1257-84B6-45F2-9ECD-DBD55820C993}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE16811-78D7-4FCE-A85D-66417DC2FE48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="10600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -398,7 +398,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CharacterHitTarget|DoDamage|BeHitCharacter|40</t>
+    <t>CharacterHitTarget|DoDamage|BeHitCharacter|18</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
Drop HP Per Second
</commit_message>
<xml_diff>
--- a/Assets/Configs/GameModifiers.xlsx
+++ b/Assets/Configs/GameModifiers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\minigame\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE16811-78D7-4FCE-A85D-66417DC2FE48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E171FC3E-A3D2-4664-B6E2-A3740244561D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="10600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="128">
   <si>
     <t>ModifierID</t>
   </si>
@@ -399,6 +399,14 @@
   </si>
   <si>
     <t>CharacterHitTarget|DoDamage|BeHitCharacter|18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>float_add|Reduce_HP_PerSecond|3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每秒掉血Buff</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -734,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="21.4140625" customWidth="1"/>
@@ -2118,6 +2126,23 @@
         <v>123</v>
       </c>
     </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>12001</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
xiu fu san she luo ji
</commit_message>
<xml_diff>
--- a/Assets/Configs/GameModifiers.xlsx
+++ b/Assets/Configs/GameModifiers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\minigame\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9998AD57-08CA-476C-A5F4-26645839CBE9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AA9BEE-7B92-40F1-BAAA-2FB0633B94D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="9570" xr2:uid="{478B3112-DF2F-4443-9DAF-B778DD3194E3}"/>
   </bookViews>
@@ -534,11 +534,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>int_set|myAttackSkillID|10</t>
+    <t>CharacterCastSkill|DispelModifier|16001|MainCharacter</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CharacterCastSkill|DispelModifier|16001|MainCharacter</t>
+    <t>int_set|myAttackSkillID|5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2350,7 +2350,7 @@
         <v>5</v>
       </c>
       <c r="D85" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E85" t="s">
         <v>131</v>
@@ -2690,7 +2690,7 @@
         <v>32</v>
       </c>
       <c r="D105" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E105" t="s">
         <v>112</v>

</xml_diff>

<commit_message>
new updates for waves and champions
</commit_message>
<xml_diff>
--- a/Assets/Configs/GameModifiers.xlsx
+++ b/Assets/Configs/GameModifiers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\minigame\Project3D\Assets\Configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AA9BEE-7B92-40F1-BAAA-2FB0633B94D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E10E40-E171-4D26-8F8D-39362ACC4F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="9570" xr2:uid="{478B3112-DF2F-4443-9DAF-B778DD3194E3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{478B3112-DF2F-4443-9DAF-B778DD3194E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -402,33 +402,15 @@
     <t>烹饪中，设置特效</t>
   </si>
   <si>
-    <t>float_add|Reduce_MP_PerSecond|3</t>
-  </si>
-  <si>
-    <t>float_add|Reduce_MP_PerSecond|1.5</t>
-  </si>
-  <si>
-    <t>基础塔：每秒消耗1.5点MP</t>
-  </si>
-  <si>
     <t>int_set|myAttackSkillID|5</t>
   </si>
   <si>
     <t>基础塔：设置攻击技能为生成子弹</t>
   </si>
   <si>
-    <t>散射塔：每秒消耗3点MP（加倍）</t>
-  </si>
-  <si>
     <t>散射塔：设置攻击技能为散射攻击</t>
   </si>
   <si>
-    <t>float_add|Reduce_MP_PerSecond|0.75</t>
-  </si>
-  <si>
-    <t>减速塔：每秒消耗0.75点MP（减半）</t>
-  </si>
-  <si>
     <t>减速塔：设置攻击技能为减速攻击</t>
   </si>
   <si>
@@ -442,9 +424,6 @@
   </si>
   <si>
     <t>散射攻击：技能使用后驱散</t>
-  </si>
-  <si>
-    <t>float_add|Reduce_MP_PerSecond|-30</t>
   </si>
   <si>
     <t>每秒回血Buff</t>
@@ -539,6 +518,138 @@
   </si>
   <si>
     <t>int_set|myAttackSkillID|5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>float_add|Reduce_MP_PerSecond|1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>float_add|Reduce_MP_PerSecond|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>float_add|Reduce_MP_PerSecond|0.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>5</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>基</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>础</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>塔：每秒消耗1点MP</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>散射塔：每秒消耗</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>点MP（加倍）</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>减速塔：每秒消耗0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>点MP（减半）</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>float_add|Reduce_MP_PerSecond|-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>50</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -546,21 +657,42 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -607,9 +739,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -647,7 +779,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -753,7 +885,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -895,7 +1027,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -904,14 +1036,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F163EA-9459-48C1-AF83-EE818DD292D1}">
   <dimension ref="A1:E110"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="3" width="22.4140625" customWidth="1"/>
-    <col min="4" max="4" width="80.58203125" customWidth="1"/>
-    <col min="5" max="5" width="22.4140625" customWidth="1"/>
+    <col min="1" max="3" width="22.3984375" customWidth="1"/>
+    <col min="4" max="4" width="80.59765625" customWidth="1"/>
+    <col min="5" max="5" width="22.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +1060,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -945,7 +1077,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -962,7 +1094,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>1</v>
       </c>
@@ -979,7 +1111,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>1</v>
       </c>
@@ -996,7 +1128,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1013,7 +1145,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1030,7 +1162,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1047,7 +1179,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1064,7 +1196,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1081,7 +1213,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1098,7 +1230,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>4</v>
       </c>
@@ -1115,7 +1247,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>5</v>
       </c>
@@ -1132,7 +1264,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>2001</v>
       </c>
@@ -1149,7 +1281,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>2001</v>
       </c>
@@ -1166,7 +1298,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>2001</v>
       </c>
@@ -1183,7 +1315,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5">
       <c r="A17">
         <v>1001</v>
       </c>
@@ -1200,7 +1332,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18">
         <v>1001</v>
       </c>
@@ -1217,7 +1349,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19">
         <v>1001</v>
       </c>
@@ -1234,7 +1366,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20">
         <v>1001</v>
       </c>
@@ -1251,7 +1383,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5">
       <c r="A21">
         <v>1001</v>
       </c>
@@ -1268,7 +1400,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5">
       <c r="A22">
         <v>1001</v>
       </c>
@@ -1285,7 +1417,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5">
       <c r="A23">
         <v>1001</v>
       </c>
@@ -1302,7 +1434,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5">
       <c r="A24">
         <v>1001</v>
       </c>
@@ -1319,7 +1451,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5">
       <c r="A25">
         <v>1001</v>
       </c>
@@ -1336,7 +1468,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5">
       <c r="A26">
         <v>1002</v>
       </c>
@@ -1353,7 +1485,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5">
       <c r="A27">
         <v>1002</v>
       </c>
@@ -1370,7 +1502,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5">
       <c r="A28">
         <v>1002</v>
       </c>
@@ -1387,7 +1519,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5">
       <c r="A29">
         <v>1002</v>
       </c>
@@ -1404,7 +1536,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5">
       <c r="A30">
         <v>1002</v>
       </c>
@@ -1421,7 +1553,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5">
       <c r="A31">
         <v>1002</v>
       </c>
@@ -1438,7 +1570,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5">
       <c r="A32">
         <v>1002</v>
       </c>
@@ -1455,7 +1587,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33">
         <v>1002</v>
       </c>
@@ -1472,7 +1604,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34">
         <v>1002</v>
       </c>
@@ -1489,7 +1621,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35">
         <v>1002</v>
       </c>
@@ -1506,7 +1638,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36">
         <v>1002</v>
       </c>
@@ -1523,7 +1655,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37">
         <v>1003</v>
       </c>
@@ -1540,7 +1672,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5">
       <c r="A38">
         <v>1003</v>
       </c>
@@ -1557,7 +1689,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5">
       <c r="A39">
         <v>1003</v>
       </c>
@@ -1574,7 +1706,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5">
       <c r="A40">
         <v>1003</v>
       </c>
@@ -1591,7 +1723,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5">
       <c r="A41">
         <v>1003</v>
       </c>
@@ -1608,7 +1740,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5">
       <c r="A42">
         <v>1003</v>
       </c>
@@ -1625,7 +1757,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5">
       <c r="A43">
         <v>1003</v>
       </c>
@@ -1642,7 +1774,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5">
       <c r="A44">
         <v>1003</v>
       </c>
@@ -1659,7 +1791,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5">
       <c r="A45">
         <v>1003</v>
       </c>
@@ -1676,7 +1808,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5">
       <c r="A46">
         <v>1003</v>
       </c>
@@ -1693,7 +1825,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5">
       <c r="A47">
         <v>1003</v>
       </c>
@@ -1710,7 +1842,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5">
       <c r="A48">
         <v>1004</v>
       </c>
@@ -1727,7 +1859,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5">
       <c r="A49">
         <v>1004</v>
       </c>
@@ -1744,7 +1876,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5">
       <c r="A50">
         <v>1004</v>
       </c>
@@ -1761,7 +1893,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5">
       <c r="A51">
         <v>1004</v>
       </c>
@@ -1778,7 +1910,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5">
       <c r="A52">
         <v>1004</v>
       </c>
@@ -1795,7 +1927,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5">
       <c r="A53">
         <v>1004</v>
       </c>
@@ -1812,7 +1944,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5">
       <c r="A54">
         <v>1004</v>
       </c>
@@ -1829,7 +1961,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5">
       <c r="A55">
         <v>1004</v>
       </c>
@@ -1846,7 +1978,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5">
       <c r="A56">
         <v>3001</v>
       </c>
@@ -1863,7 +1995,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5">
       <c r="A57">
         <v>3001</v>
       </c>
@@ -1874,13 +2006,13 @@
         <v>32</v>
       </c>
       <c r="D57" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="E57" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5">
       <c r="A58">
         <v>3001</v>
       </c>
@@ -1897,7 +2029,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5">
       <c r="A59">
         <v>3002</v>
       </c>
@@ -1914,7 +2046,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5">
       <c r="A60">
         <v>3002</v>
       </c>
@@ -1931,7 +2063,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5">
       <c r="A61">
         <v>3002</v>
       </c>
@@ -1948,7 +2080,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5">
       <c r="A62">
         <v>4001</v>
       </c>
@@ -1965,7 +2097,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5">
       <c r="A63">
         <v>4001</v>
       </c>
@@ -1982,7 +2114,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5">
       <c r="A64">
         <v>4002</v>
       </c>
@@ -1999,7 +2131,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5">
       <c r="A65">
         <v>4002</v>
       </c>
@@ -2016,7 +2148,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5">
       <c r="A66">
         <v>4002</v>
       </c>
@@ -2033,7 +2165,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5">
       <c r="A67">
         <v>4002</v>
       </c>
@@ -2050,7 +2182,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5">
       <c r="A68">
         <v>5001</v>
       </c>
@@ -2067,7 +2199,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5">
       <c r="A69">
         <v>5001</v>
       </c>
@@ -2084,7 +2216,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5">
       <c r="A70">
         <v>6001</v>
       </c>
@@ -2101,7 +2233,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5">
       <c r="A71">
         <v>6001</v>
       </c>
@@ -2118,7 +2250,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5">
       <c r="A72">
         <v>7001</v>
       </c>
@@ -2135,7 +2267,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5">
       <c r="A73">
         <v>7001</v>
       </c>
@@ -2152,7 +2284,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5">
       <c r="A74">
         <v>8001</v>
       </c>
@@ -2169,7 +2301,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5">
       <c r="A75">
         <v>8001</v>
       </c>
@@ -2186,7 +2318,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5">
       <c r="A76">
         <v>8001</v>
       </c>
@@ -2203,7 +2335,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5">
       <c r="A77">
         <v>9001</v>
       </c>
@@ -2220,7 +2352,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5">
       <c r="A78">
         <v>9001</v>
       </c>
@@ -2237,7 +2369,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5">
       <c r="A79">
         <v>10001</v>
       </c>
@@ -2254,7 +2386,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5">
       <c r="A80">
         <v>10001</v>
       </c>
@@ -2271,7 +2403,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5">
       <c r="A81">
         <v>11001</v>
       </c>
@@ -2288,7 +2420,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5">
       <c r="A82">
         <v>12001</v>
       </c>
@@ -2299,13 +2431,13 @@
         <v>5</v>
       </c>
       <c r="D82" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="E82" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
       <c r="A83">
         <v>12001</v>
       </c>
@@ -2316,13 +2448,13 @@
         <v>5</v>
       </c>
       <c r="D83" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E83" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
       <c r="A84">
         <v>12002</v>
       </c>
@@ -2333,13 +2465,13 @@
         <v>5</v>
       </c>
       <c r="D84" t="s">
-        <v>125</v>
+        <v>162</v>
       </c>
       <c r="E84" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
       <c r="A85">
         <v>12002</v>
       </c>
@@ -2350,13 +2482,13 @@
         <v>5</v>
       </c>
       <c r="D85" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E85" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
       <c r="A86">
         <v>12003</v>
       </c>
@@ -2367,13 +2499,13 @@
         <v>5</v>
       </c>
       <c r="D86" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="E86" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
       <c r="A87">
         <v>12003</v>
       </c>
@@ -2384,13 +2516,13 @@
         <v>5</v>
       </c>
       <c r="D87" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="E87" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
       <c r="A88">
         <v>13001</v>
       </c>
@@ -2401,13 +2533,13 @@
         <v>32</v>
       </c>
       <c r="D88" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E88" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
       <c r="A89">
         <v>13001</v>
       </c>
@@ -2418,13 +2550,13 @@
         <v>32</v>
       </c>
       <c r="D89" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E89" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
       <c r="A90">
         <v>13001</v>
       </c>
@@ -2435,13 +2567,13 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>139</v>
+        <v>167</v>
       </c>
       <c r="E90" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
       <c r="A91">
         <v>14001</v>
       </c>
@@ -2452,13 +2584,13 @@
         <v>32</v>
       </c>
       <c r="D91" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="E91" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
       <c r="A92">
         <v>14001</v>
       </c>
@@ -2469,13 +2601,13 @@
         <v>32</v>
       </c>
       <c r="D92" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E92" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
       <c r="A93">
         <v>14002</v>
       </c>
@@ -2486,13 +2618,13 @@
         <v>32</v>
       </c>
       <c r="D93" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="E93" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
       <c r="A94">
         <v>14002</v>
       </c>
@@ -2503,13 +2635,13 @@
         <v>32</v>
       </c>
       <c r="D94" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E94" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
       <c r="A95">
         <v>15001</v>
       </c>
@@ -2520,13 +2652,13 @@
         <v>5</v>
       </c>
       <c r="D95" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E95" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
       <c r="A96">
         <v>15001</v>
       </c>
@@ -2537,13 +2669,13 @@
         <v>12</v>
       </c>
       <c r="D96" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="E96" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
       <c r="A97">
         <v>8002</v>
       </c>
@@ -2560,7 +2692,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5">
       <c r="A98">
         <v>8002</v>
       </c>
@@ -2571,13 +2703,13 @@
         <v>32</v>
       </c>
       <c r="D98" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E98" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
       <c r="A99">
         <v>8002</v>
       </c>
@@ -2594,7 +2726,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5">
       <c r="A100">
         <v>8003</v>
       </c>
@@ -2611,7 +2743,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5">
       <c r="A101">
         <v>8003</v>
       </c>
@@ -2622,13 +2754,13 @@
         <v>32</v>
       </c>
       <c r="D101" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E101" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
       <c r="A102">
         <v>8003</v>
       </c>
@@ -2645,7 +2777,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5">
       <c r="A103">
         <v>12004</v>
       </c>
@@ -2656,13 +2788,13 @@
         <v>5</v>
       </c>
       <c r="D103" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="E103" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
       <c r="A104">
         <v>16001</v>
       </c>
@@ -2673,13 +2805,13 @@
         <v>32</v>
       </c>
       <c r="D104" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="E104" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5">
       <c r="A105">
         <v>16001</v>
       </c>
@@ -2690,13 +2822,13 @@
         <v>32</v>
       </c>
       <c r="D105" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="E105" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5">
       <c r="A106">
         <v>16002</v>
       </c>
@@ -2707,13 +2839,13 @@
         <v>5</v>
       </c>
       <c r="D106" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="E106" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5">
       <c r="A107">
         <v>16002</v>
       </c>
@@ -2724,13 +2856,13 @@
         <v>32</v>
       </c>
       <c r="D107" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="E107" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5">
       <c r="A108">
         <v>16002</v>
       </c>
@@ -2741,13 +2873,13 @@
         <v>32</v>
       </c>
       <c r="D108" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="E108" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5">
       <c r="A109">
         <v>16002</v>
       </c>
@@ -2764,7 +2896,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5">
       <c r="A110">
         <v>16003</v>
       </c>
@@ -2775,10 +2907,10 @@
         <v>5</v>
       </c>
       <c r="D110" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E110" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new updates for bullets and waves
</commit_message>
<xml_diff>
--- a/Assets/Configs/GameModifiers.xlsx
+++ b/Assets/Configs/GameModifiers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E10E40-E171-4D26-8F8D-39362ACC4F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E3FA3A-0F4A-45C8-AF4F-DDCD937DC092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{478B3112-DF2F-4443-9DAF-B778DD3194E3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="170">
   <si>
     <t>ModifierID</t>
   </si>
@@ -388,9 +388,6 @@
   </si>
   <si>
     <t>CharacterCastSkill|DispelModifier|9001|MainCharacter</t>
-  </si>
-  <si>
-    <t>CharacterCastSkill|DropCurObject|MainCharacter</t>
   </si>
   <si>
     <t>放下手里的物品</t>
@@ -498,10 +495,6 @@
   </si>
   <si>
     <t>CharacterHitTarget|AddModifier|16003|BeHitCharacter|1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>float_add|MaxSpeed|-0.5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -650,6 +643,46 @@
       </rPr>
       <t>50</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>float_add|MaxSpeed|-0.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>25</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharacterCastSkill|DropCurObject|MainCharacter</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>CharacterHitTarget|DoDamage|BeHitCharacter|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>36</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharacterHitTarget|DoDamage|DoHitCharacter|9999</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2006,7 +2039,7 @@
         <v>32</v>
       </c>
       <c r="D57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E57" t="s">
         <v>84</v>
@@ -2380,10 +2413,10 @@
         <v>32</v>
       </c>
       <c r="D79" t="s">
+        <v>167</v>
+      </c>
+      <c r="E79" t="s">
         <v>121</v>
-      </c>
-      <c r="E79" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -2397,10 +2430,10 @@
         <v>32</v>
       </c>
       <c r="D80" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E80" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -2417,7 +2450,7 @@
         <v>13</v>
       </c>
       <c r="E81" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -2431,10 +2464,10 @@
         <v>5</v>
       </c>
       <c r="D82" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E82" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -2448,10 +2481,10 @@
         <v>5</v>
       </c>
       <c r="D83" t="s">
+        <v>124</v>
+      </c>
+      <c r="E83" t="s">
         <v>125</v>
-      </c>
-      <c r="E83" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -2465,10 +2498,10 @@
         <v>5</v>
       </c>
       <c r="D84" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E84" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -2482,10 +2515,10 @@
         <v>5</v>
       </c>
       <c r="D85" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E85" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -2499,10 +2532,10 @@
         <v>5</v>
       </c>
       <c r="D86" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E86" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -2516,10 +2549,10 @@
         <v>5</v>
       </c>
       <c r="D87" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E87" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -2533,10 +2566,10 @@
         <v>32</v>
       </c>
       <c r="D88" t="s">
+        <v>128</v>
+      </c>
+      <c r="E88" t="s">
         <v>129</v>
-      </c>
-      <c r="E88" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -2550,10 +2583,10 @@
         <v>32</v>
       </c>
       <c r="D89" t="s">
+        <v>130</v>
+      </c>
+      <c r="E89" t="s">
         <v>131</v>
-      </c>
-      <c r="E89" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -2567,10 +2600,10 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E90" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -2584,10 +2617,10 @@
         <v>32</v>
       </c>
       <c r="D91" t="s">
+        <v>133</v>
+      </c>
+      <c r="E91" t="s">
         <v>134</v>
-      </c>
-      <c r="E91" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -2601,10 +2634,10 @@
         <v>32</v>
       </c>
       <c r="D92" t="s">
+        <v>135</v>
+      </c>
+      <c r="E92" t="s">
         <v>136</v>
-      </c>
-      <c r="E92" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -2618,10 +2651,10 @@
         <v>32</v>
       </c>
       <c r="D93" t="s">
+        <v>137</v>
+      </c>
+      <c r="E93" t="s">
         <v>138</v>
-      </c>
-      <c r="E93" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -2635,10 +2668,10 @@
         <v>32</v>
       </c>
       <c r="D94" t="s">
+        <v>139</v>
+      </c>
+      <c r="E94" t="s">
         <v>140</v>
-      </c>
-      <c r="E94" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -2652,10 +2685,10 @@
         <v>5</v>
       </c>
       <c r="D95" t="s">
+        <v>141</v>
+      </c>
+      <c r="E95" t="s">
         <v>142</v>
-      </c>
-      <c r="E95" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -2669,10 +2702,10 @@
         <v>12</v>
       </c>
       <c r="D96" t="s">
+        <v>143</v>
+      </c>
+      <c r="E96" t="s">
         <v>144</v>
-      </c>
-      <c r="E96" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2703,10 +2736,10 @@
         <v>32</v>
       </c>
       <c r="D98" t="s">
+        <v>145</v>
+      </c>
+      <c r="E98" t="s">
         <v>146</v>
-      </c>
-      <c r="E98" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2754,10 +2787,10 @@
         <v>32</v>
       </c>
       <c r="D101" t="s">
+        <v>168</v>
+      </c>
+      <c r="E101" t="s">
         <v>146</v>
-      </c>
-      <c r="E101" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2771,7 +2804,7 @@
         <v>32</v>
       </c>
       <c r="D102" t="s">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="E102" t="s">
         <v>118</v>
@@ -2788,10 +2821,10 @@
         <v>5</v>
       </c>
       <c r="D103" t="s">
+        <v>147</v>
+      </c>
+      <c r="E103" t="s">
         <v>148</v>
-      </c>
-      <c r="E103" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2805,7 +2838,7 @@
         <v>32</v>
       </c>
       <c r="D104" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E104" t="s">
         <v>110</v>
@@ -2822,7 +2855,7 @@
         <v>32</v>
       </c>
       <c r="D105" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E105" t="s">
         <v>112</v>
@@ -2839,7 +2872,7 @@
         <v>5</v>
       </c>
       <c r="D106" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E106" t="s">
         <v>114</v>
@@ -2856,7 +2889,7 @@
         <v>32</v>
       </c>
       <c r="D107" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E107" t="s">
         <v>116</v>
@@ -2873,10 +2906,10 @@
         <v>32</v>
       </c>
       <c r="D108" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E108" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2907,10 +2940,10 @@
         <v>5</v>
       </c>
       <c r="D110" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="E110" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>